<commit_message>
feat(import): cantidad de slides para Carrusel (selector + plantilla + agente)
</commit_message>
<xml_diff>
--- a/src/assets/plantilla-plan-windstudies.xlsx
+++ b/src/assets/plantilla-plan-windstudies.xlsx
@@ -678,6 +678,11 @@
       </c>
       <c r="I5" s="7" t="s">
         <v>14</v>
+      </c>
+      <c r="J5" s="7" t="inlineStr">
+        <is>
+          <t>Cantidad de Slides</t>
+        </is>
       </c>
     </row>
     <row r="6" ht="21.75" customHeight="1">
@@ -1963,7 +1968,7 @@
     <mergeCell ref="A3:I3"/>
   </mergeCells>
   <printOptions/>
-  <dataValidations count="4">
+  <dataValidations count="5">
     <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="D6:D105">
       <formula1>"Reel,Post,Story,Carrusel"</formula1>
     </dataValidation>
@@ -1975,6 +1980,9 @@
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="G6:G105">
       <formula1>"1,2,3,4,5"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="J6:J105">
+      <formula1>"3,4,5,6,7,8,9,10"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins bottom="1.0" footer="0.0" header="0.0" left="0.75" right="0.75" top="1.0"/>
@@ -2067,6 +2075,11 @@
       </c>
       <c r="I5" s="7" t="s">
         <v>14</v>
+      </c>
+      <c r="J5" s="7" t="inlineStr">
+        <is>
+          <t>Cantidad de Slides</t>
+        </is>
       </c>
     </row>
     <row r="6" ht="21.75" customHeight="1">
@@ -3352,7 +3365,7 @@
     <mergeCell ref="A3:I3"/>
   </mergeCells>
   <printOptions/>
-  <dataValidations count="4">
+  <dataValidations count="5">
     <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="D6:D105">
       <formula1>"Reel,Post,Story,Carrusel"</formula1>
     </dataValidation>
@@ -3364,6 +3377,9 @@
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="G6:G105">
       <formula1>"1,2,3,4,5"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="J6:J105">
+      <formula1>"3,4,5,6,7,8,9,10"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins bottom="1.0" footer="0.0" header="0.0" left="0.75" right="0.75" top="1.0"/>
@@ -3456,6 +3472,11 @@
       </c>
       <c r="I5" s="7" t="s">
         <v>14</v>
+      </c>
+      <c r="J5" s="7" t="inlineStr">
+        <is>
+          <t>Cantidad de Slides</t>
+        </is>
       </c>
     </row>
     <row r="6" ht="21.75" customHeight="1">
@@ -4741,7 +4762,7 @@
     <mergeCell ref="A3:I3"/>
   </mergeCells>
   <printOptions/>
-  <dataValidations count="4">
+  <dataValidations count="5">
     <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="D6:D105">
       <formula1>"Reel,Post,Story,Carrusel"</formula1>
     </dataValidation>
@@ -4753,6 +4774,9 @@
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="G6:G105">
       <formula1>"1,2,3,4,5"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="J6:J105">
+      <formula1>"3,4,5,6,7,8,9,10"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins bottom="1.0" footer="0.0" header="0.0" left="0.75" right="0.75" top="1.0"/>
@@ -4845,6 +4869,11 @@
       </c>
       <c r="I5" s="7" t="s">
         <v>14</v>
+      </c>
+      <c r="J5" s="7" t="inlineStr">
+        <is>
+          <t>Cantidad de Slides</t>
+        </is>
       </c>
     </row>
     <row r="6" ht="21.75" customHeight="1">
@@ -6130,7 +6159,7 @@
     <mergeCell ref="A3:I3"/>
   </mergeCells>
   <printOptions/>
-  <dataValidations count="4">
+  <dataValidations count="5">
     <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="D6:D105">
       <formula1>"Reel,Post,Story,Carrusel"</formula1>
     </dataValidation>
@@ -6142,6 +6171,9 @@
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="G6:G105">
       <formula1>"1,2,3,4,5"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="J6:J105">
+      <formula1>"3,4,5,6,7,8,9,10"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins bottom="1.0" footer="0.0" header="0.0" left="0.75" right="0.75" top="1.0"/>
@@ -6234,6 +6266,11 @@
       </c>
       <c r="I5" s="7" t="s">
         <v>14</v>
+      </c>
+      <c r="J5" s="7" t="inlineStr">
+        <is>
+          <t>Cantidad de Slides</t>
+        </is>
       </c>
     </row>
     <row r="6" ht="21.75" customHeight="1">
@@ -7310,7 +7347,7 @@
     <mergeCell ref="A3:I3"/>
   </mergeCells>
   <printOptions/>
-  <dataValidations count="4">
+  <dataValidations count="5">
     <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="D6:D105">
       <formula1>"Reel,Post,Story,Carrusel"</formula1>
     </dataValidation>
@@ -7323,6 +7360,9 @@
     <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="G6:G105">
       <formula1>"1,2,3,4,5"</formula1>
     </dataValidation>
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="J6:J105">
+      <formula1>"3,4,5,6,7,8,9,10"</formula1>
+    </dataValidation>
   </dataValidations>
   <pageMargins bottom="1.0" footer="0.0" header="0.0" left="0.75" right="0.75" top="1.0"/>
   <pageSetup orientation="landscape"/>

</xml_diff>

<commit_message>
feat(import): tipo de reel y tipo de carrusel (selectores + plantilla + agente)
</commit_message>
<xml_diff>
--- a/src/assets/plantilla-plan-windstudies.xlsx
+++ b/src/assets/plantilla-plan-windstudies.xlsx
@@ -682,6 +682,16 @@
       <c r="J5" s="7" t="inlineStr">
         <is>
           <t>Cantidad de Slides</t>
+        </is>
+      </c>
+      <c r="K5" s="7" t="inlineStr">
+        <is>
+          <t>Tipo de Reel</t>
+        </is>
+      </c>
+      <c r="L5" s="7" t="inlineStr">
+        <is>
+          <t>Tipo de Carrusel</t>
         </is>
       </c>
     </row>
@@ -1968,7 +1978,7 @@
     <mergeCell ref="A3:I3"/>
   </mergeCells>
   <printOptions/>
-  <dataValidations count="5">
+  <dataValidations count="7">
     <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="D6:D105">
       <formula1>"Reel,Post,Story,Carrusel"</formula1>
     </dataValidation>
@@ -1983,6 +1993,12 @@
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="J6:J105">
       <formula1>"3,4,5,6,7,8,9,10"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="K6:K105">
+      <formula1>"Talking head,UGC / testimonio,Tutorial / educativo,Trend / audio viral"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="L6:L105">
+      <formula1>"Educativo / tips,Storytelling,Antes / después,Listicle"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins bottom="1.0" footer="0.0" header="0.0" left="0.75" right="0.75" top="1.0"/>
@@ -2079,6 +2095,16 @@
       <c r="J5" s="7" t="inlineStr">
         <is>
           <t>Cantidad de Slides</t>
+        </is>
+      </c>
+      <c r="K5" s="7" t="inlineStr">
+        <is>
+          <t>Tipo de Reel</t>
+        </is>
+      </c>
+      <c r="L5" s="7" t="inlineStr">
+        <is>
+          <t>Tipo de Carrusel</t>
         </is>
       </c>
     </row>
@@ -3365,7 +3391,7 @@
     <mergeCell ref="A3:I3"/>
   </mergeCells>
   <printOptions/>
-  <dataValidations count="5">
+  <dataValidations count="7">
     <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="D6:D105">
       <formula1>"Reel,Post,Story,Carrusel"</formula1>
     </dataValidation>
@@ -3380,6 +3406,12 @@
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="J6:J105">
       <formula1>"3,4,5,6,7,8,9,10"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="K6:K105">
+      <formula1>"Talking head,UGC / testimonio,Tutorial / educativo,Trend / audio viral"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="L6:L105">
+      <formula1>"Educativo / tips,Storytelling,Antes / después,Listicle"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins bottom="1.0" footer="0.0" header="0.0" left="0.75" right="0.75" top="1.0"/>
@@ -3476,6 +3508,16 @@
       <c r="J5" s="7" t="inlineStr">
         <is>
           <t>Cantidad de Slides</t>
+        </is>
+      </c>
+      <c r="K5" s="7" t="inlineStr">
+        <is>
+          <t>Tipo de Reel</t>
+        </is>
+      </c>
+      <c r="L5" s="7" t="inlineStr">
+        <is>
+          <t>Tipo de Carrusel</t>
         </is>
       </c>
     </row>
@@ -4762,7 +4804,7 @@
     <mergeCell ref="A3:I3"/>
   </mergeCells>
   <printOptions/>
-  <dataValidations count="5">
+  <dataValidations count="7">
     <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="D6:D105">
       <formula1>"Reel,Post,Story,Carrusel"</formula1>
     </dataValidation>
@@ -4777,6 +4819,12 @@
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="J6:J105">
       <formula1>"3,4,5,6,7,8,9,10"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="K6:K105">
+      <formula1>"Talking head,UGC / testimonio,Tutorial / educativo,Trend / audio viral"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="L6:L105">
+      <formula1>"Educativo / tips,Storytelling,Antes / después,Listicle"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins bottom="1.0" footer="0.0" header="0.0" left="0.75" right="0.75" top="1.0"/>
@@ -4873,6 +4921,16 @@
       <c r="J5" s="7" t="inlineStr">
         <is>
           <t>Cantidad de Slides</t>
+        </is>
+      </c>
+      <c r="K5" s="7" t="inlineStr">
+        <is>
+          <t>Tipo de Reel</t>
+        </is>
+      </c>
+      <c r="L5" s="7" t="inlineStr">
+        <is>
+          <t>Tipo de Carrusel</t>
         </is>
       </c>
     </row>
@@ -6159,7 +6217,7 @@
     <mergeCell ref="A3:I3"/>
   </mergeCells>
   <printOptions/>
-  <dataValidations count="5">
+  <dataValidations count="7">
     <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="D6:D105">
       <formula1>"Reel,Post,Story,Carrusel"</formula1>
     </dataValidation>
@@ -6174,6 +6232,12 @@
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="J6:J105">
       <formula1>"3,4,5,6,7,8,9,10"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="K6:K105">
+      <formula1>"Talking head,UGC / testimonio,Tutorial / educativo,Trend / audio viral"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="L6:L105">
+      <formula1>"Educativo / tips,Storytelling,Antes / después,Listicle"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins bottom="1.0" footer="0.0" header="0.0" left="0.75" right="0.75" top="1.0"/>
@@ -6270,6 +6334,16 @@
       <c r="J5" s="7" t="inlineStr">
         <is>
           <t>Cantidad de Slides</t>
+        </is>
+      </c>
+      <c r="K5" s="7" t="inlineStr">
+        <is>
+          <t>Tipo de Reel</t>
+        </is>
+      </c>
+      <c r="L5" s="7" t="inlineStr">
+        <is>
+          <t>Tipo de Carrusel</t>
         </is>
       </c>
     </row>
@@ -7347,7 +7421,7 @@
     <mergeCell ref="A3:I3"/>
   </mergeCells>
   <printOptions/>
-  <dataValidations count="5">
+  <dataValidations count="7">
     <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="D6:D105">
       <formula1>"Reel,Post,Story,Carrusel"</formula1>
     </dataValidation>
@@ -7363,6 +7437,12 @@
     <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="J6:J105">
       <formula1>"3,4,5,6,7,8,9,10"</formula1>
     </dataValidation>
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="K6:K105">
+      <formula1>"Talking head,UGC / testimonio,Tutorial / educativo,Trend / audio viral"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="L6:L105">
+      <formula1>"Educativo / tips,Storytelling,Antes / después,Listicle"</formula1>
+    </dataValidation>
   </dataValidations>
   <pageMargins bottom="1.0" footer="0.0" header="0.0" left="0.75" right="0.75" top="1.0"/>
   <pageSetup orientation="landscape"/>

</xml_diff>

<commit_message>
feat(plantilla): columnas de tipo agrupadas junto a TIPO DE STORY, en mayúscula; preview alineado
</commit_message>
<xml_diff>
--- a/src/assets/plantilla-plan-windstudies.xlsx
+++ b/src/assets/plantilla-plan-windstudies.xlsx
@@ -607,10 +607,13 @@
     <col customWidth="1" min="4" max="4" width="13.0"/>
     <col customWidth="1" min="5" max="5" width="11.0"/>
     <col customWidth="1" min="6" max="6" width="17.0"/>
-    <col customWidth="1" min="7" max="7" width="8.0"/>
-    <col customWidth="1" min="8" max="8" width="13.0"/>
-    <col customWidth="1" min="9" max="9" width="36.0"/>
-    <col customWidth="1" min="10" max="26" width="8.71"/>
+    <col customWidth="1" min="7" max="7" width="17.0"/>
+    <col customWidth="1" min="8" max="8" width="17.0"/>
+    <col customWidth="1" min="9" max="9" width="13.0"/>
+    <col customWidth="1" min="10" max="10" width="8.0"/>
+    <col customWidth="1" min="11" max="11" width="10.0"/>
+    <col customWidth="1" min="12" max="12" width="36.0"/>
+    <col min="13" max="26" width="9.0"/>
   </cols>
   <sheetData>
     <row r="1" ht="30.0" customHeight="1">
@@ -652,46 +655,64 @@
     </row>
     <row r="4" ht="6.0" customHeight="1"/>
     <row r="5" ht="27.75" customHeight="1">
-      <c r="A5" s="7" t="s">
-        <v>6</v>
-      </c>
-      <c r="B5" s="7" t="s">
-        <v>7</v>
-      </c>
-      <c r="C5" s="7" t="s">
-        <v>8</v>
-      </c>
-      <c r="D5" s="7" t="s">
-        <v>9</v>
-      </c>
-      <c r="E5" s="7" t="s">
-        <v>10</v>
-      </c>
-      <c r="F5" s="7" t="s">
-        <v>11</v>
-      </c>
-      <c r="G5" s="7" t="s">
-        <v>12</v>
-      </c>
-      <c r="H5" s="7" t="s">
-        <v>13</v>
-      </c>
-      <c r="I5" s="7" t="s">
-        <v>14</v>
+      <c r="A5" s="7" t="inlineStr">
+        <is>
+          <t>DÍA</t>
+        </is>
+      </c>
+      <c r="B5" s="7" t="inlineStr">
+        <is>
+          <t>FECHA DE PUBLICACIÓN</t>
+        </is>
+      </c>
+      <c r="C5" s="7" t="inlineStr">
+        <is>
+          <t>N°</t>
+        </is>
+      </c>
+      <c r="D5" s="7" t="inlineStr">
+        <is>
+          <t>TIPO DE PIEZA</t>
+        </is>
+      </c>
+      <c r="E5" s="7" t="inlineStr">
+        <is>
+          <t>DURACIÓN</t>
+        </is>
+      </c>
+      <c r="F5" s="7" t="inlineStr">
+        <is>
+          <t>TIPO DE STORY</t>
+        </is>
+      </c>
+      <c r="G5" s="7" t="inlineStr">
+        <is>
+          <t>TIPO DE REEL</t>
+        </is>
+      </c>
+      <c r="H5" s="7" t="inlineStr">
+        <is>
+          <t>TIPO DE CARRUSEL</t>
+        </is>
+      </c>
+      <c r="I5" s="7" t="inlineStr">
+        <is>
+          <t>CANTIDAD DE SLIDES</t>
+        </is>
       </c>
       <c r="J5" s="7" t="inlineStr">
         <is>
-          <t>Cantidad de Slides</t>
+          <t>ANILLO</t>
         </is>
       </c>
       <c r="K5" s="7" t="inlineStr">
         <is>
-          <t>Tipo de Reel</t>
+          <t>PARA AD</t>
         </is>
       </c>
       <c r="L5" s="7" t="inlineStr">
         <is>
-          <t>Tipo de Carrusel</t>
+          <t>OBSERVACIONES ESTRATÉGICAS</t>
         </is>
       </c>
     </row>
@@ -1972,10 +1993,10 @@
     <row r="1000" ht="15.75" customHeight="1"/>
   </sheetData>
   <mergeCells count="4">
-    <mergeCell ref="A1:I1"/>
+    <mergeCell ref="A1:L1"/>
     <mergeCell ref="B2:D2"/>
-    <mergeCell ref="F2:I2"/>
-    <mergeCell ref="A3:I3"/>
+    <mergeCell ref="F2:L2"/>
+    <mergeCell ref="A3:L3"/>
   </mergeCells>
   <printOptions/>
   <dataValidations count="7">
@@ -1989,16 +2010,16 @@
       <formula1>"informativa,encuesta,caja_de_pregunta,micro_impacto"</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="G6:G105">
-      <formula1>"1,2,3,4,5"</formula1>
+      <formula1>"Talking head,UGC / testimonio,Tutorial / educativo,Trend / audio viral"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="H6:H105">
+      <formula1>"Educativo / tips,Storytelling,Antes / después,Listicle"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="I6:I105">
+      <formula1>"3,4,5,6,7,8,9,10"</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="J6:J105">
-      <formula1>"3,4,5,6,7,8,9,10"</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="K6:K105">
-      <formula1>"Talking head,UGC / testimonio,Tutorial / educativo,Trend / audio viral"</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="L6:L105">
-      <formula1>"Educativo / tips,Storytelling,Antes / después,Listicle"</formula1>
+      <formula1>"1,2,3,4,5"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins bottom="1.0" footer="0.0" header="0.0" left="0.75" right="0.75" top="1.0"/>
@@ -2020,10 +2041,13 @@
     <col customWidth="1" min="4" max="4" width="13.0"/>
     <col customWidth="1" min="5" max="5" width="11.0"/>
     <col customWidth="1" min="6" max="6" width="17.0"/>
-    <col customWidth="1" min="7" max="7" width="8.0"/>
-    <col customWidth="1" min="8" max="8" width="13.0"/>
-    <col customWidth="1" min="9" max="9" width="36.0"/>
-    <col customWidth="1" min="10" max="26" width="8.71"/>
+    <col customWidth="1" min="7" max="7" width="17.0"/>
+    <col customWidth="1" min="8" max="8" width="17.0"/>
+    <col customWidth="1" min="9" max="9" width="13.0"/>
+    <col customWidth="1" min="10" max="10" width="8.0"/>
+    <col customWidth="1" min="11" max="11" width="10.0"/>
+    <col customWidth="1" min="12" max="12" width="36.0"/>
+    <col min="13" max="26" width="9.0"/>
   </cols>
   <sheetData>
     <row r="1" ht="30.0" customHeight="1">
@@ -2065,46 +2089,64 @@
     </row>
     <row r="4" ht="6.0" customHeight="1"/>
     <row r="5" ht="27.75" customHeight="1">
-      <c r="A5" s="7" t="s">
-        <v>6</v>
-      </c>
-      <c r="B5" s="7" t="s">
-        <v>7</v>
-      </c>
-      <c r="C5" s="7" t="s">
-        <v>8</v>
-      </c>
-      <c r="D5" s="7" t="s">
-        <v>9</v>
-      </c>
-      <c r="E5" s="7" t="s">
-        <v>10</v>
-      </c>
-      <c r="F5" s="7" t="s">
-        <v>11</v>
-      </c>
-      <c r="G5" s="7" t="s">
-        <v>12</v>
-      </c>
-      <c r="H5" s="7" t="s">
-        <v>13</v>
-      </c>
-      <c r="I5" s="7" t="s">
-        <v>14</v>
+      <c r="A5" s="7" t="inlineStr">
+        <is>
+          <t>DÍA</t>
+        </is>
+      </c>
+      <c r="B5" s="7" t="inlineStr">
+        <is>
+          <t>FECHA DE PUBLICACIÓN</t>
+        </is>
+      </c>
+      <c r="C5" s="7" t="inlineStr">
+        <is>
+          <t>N°</t>
+        </is>
+      </c>
+      <c r="D5" s="7" t="inlineStr">
+        <is>
+          <t>TIPO DE PIEZA</t>
+        </is>
+      </c>
+      <c r="E5" s="7" t="inlineStr">
+        <is>
+          <t>DURACIÓN</t>
+        </is>
+      </c>
+      <c r="F5" s="7" t="inlineStr">
+        <is>
+          <t>TIPO DE STORY</t>
+        </is>
+      </c>
+      <c r="G5" s="7" t="inlineStr">
+        <is>
+          <t>TIPO DE REEL</t>
+        </is>
+      </c>
+      <c r="H5" s="7" t="inlineStr">
+        <is>
+          <t>TIPO DE CARRUSEL</t>
+        </is>
+      </c>
+      <c r="I5" s="7" t="inlineStr">
+        <is>
+          <t>CANTIDAD DE SLIDES</t>
+        </is>
       </c>
       <c r="J5" s="7" t="inlineStr">
         <is>
-          <t>Cantidad de Slides</t>
+          <t>ANILLO</t>
         </is>
       </c>
       <c r="K5" s="7" t="inlineStr">
         <is>
-          <t>Tipo de Reel</t>
+          <t>PARA AD</t>
         </is>
       </c>
       <c r="L5" s="7" t="inlineStr">
         <is>
-          <t>Tipo de Carrusel</t>
+          <t>OBSERVACIONES ESTRATÉGICAS</t>
         </is>
       </c>
     </row>
@@ -3385,10 +3427,10 @@
     <row r="1000" ht="15.75" customHeight="1"/>
   </sheetData>
   <mergeCells count="4">
-    <mergeCell ref="A1:I1"/>
+    <mergeCell ref="A1:L1"/>
     <mergeCell ref="B2:D2"/>
-    <mergeCell ref="F2:I2"/>
-    <mergeCell ref="A3:I3"/>
+    <mergeCell ref="F2:L2"/>
+    <mergeCell ref="A3:L3"/>
   </mergeCells>
   <printOptions/>
   <dataValidations count="7">
@@ -3402,16 +3444,16 @@
       <formula1>"informativa,encuesta,caja_de_pregunta,micro_impacto"</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="G6:G105">
-      <formula1>"1,2,3,4,5"</formula1>
+      <formula1>"Talking head,UGC / testimonio,Tutorial / educativo,Trend / audio viral"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="H6:H105">
+      <formula1>"Educativo / tips,Storytelling,Antes / después,Listicle"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="I6:I105">
+      <formula1>"3,4,5,6,7,8,9,10"</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="J6:J105">
-      <formula1>"3,4,5,6,7,8,9,10"</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="K6:K105">
-      <formula1>"Talking head,UGC / testimonio,Tutorial / educativo,Trend / audio viral"</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="L6:L105">
-      <formula1>"Educativo / tips,Storytelling,Antes / después,Listicle"</formula1>
+      <formula1>"1,2,3,4,5"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins bottom="1.0" footer="0.0" header="0.0" left="0.75" right="0.75" top="1.0"/>
@@ -3433,10 +3475,13 @@
     <col customWidth="1" min="4" max="4" width="13.0"/>
     <col customWidth="1" min="5" max="5" width="11.0"/>
     <col customWidth="1" min="6" max="6" width="17.0"/>
-    <col customWidth="1" min="7" max="7" width="8.0"/>
-    <col customWidth="1" min="8" max="8" width="13.0"/>
-    <col customWidth="1" min="9" max="9" width="36.0"/>
-    <col customWidth="1" min="10" max="26" width="8.71"/>
+    <col customWidth="1" min="7" max="7" width="17.0"/>
+    <col customWidth="1" min="8" max="8" width="17.0"/>
+    <col customWidth="1" min="9" max="9" width="13.0"/>
+    <col customWidth="1" min="10" max="10" width="8.0"/>
+    <col customWidth="1" min="11" max="11" width="10.0"/>
+    <col customWidth="1" min="12" max="12" width="36.0"/>
+    <col min="13" max="26" width="9.0"/>
   </cols>
   <sheetData>
     <row r="1" ht="30.0" customHeight="1">
@@ -3478,46 +3523,64 @@
     </row>
     <row r="4" ht="6.0" customHeight="1"/>
     <row r="5" ht="27.75" customHeight="1">
-      <c r="A5" s="7" t="s">
-        <v>6</v>
-      </c>
-      <c r="B5" s="7" t="s">
-        <v>7</v>
-      </c>
-      <c r="C5" s="7" t="s">
-        <v>8</v>
-      </c>
-      <c r="D5" s="7" t="s">
-        <v>9</v>
-      </c>
-      <c r="E5" s="7" t="s">
-        <v>10</v>
-      </c>
-      <c r="F5" s="7" t="s">
-        <v>11</v>
-      </c>
-      <c r="G5" s="7" t="s">
-        <v>12</v>
-      </c>
-      <c r="H5" s="7" t="s">
-        <v>13</v>
-      </c>
-      <c r="I5" s="7" t="s">
-        <v>14</v>
+      <c r="A5" s="7" t="inlineStr">
+        <is>
+          <t>DÍA</t>
+        </is>
+      </c>
+      <c r="B5" s="7" t="inlineStr">
+        <is>
+          <t>FECHA DE PUBLICACIÓN</t>
+        </is>
+      </c>
+      <c r="C5" s="7" t="inlineStr">
+        <is>
+          <t>N°</t>
+        </is>
+      </c>
+      <c r="D5" s="7" t="inlineStr">
+        <is>
+          <t>TIPO DE PIEZA</t>
+        </is>
+      </c>
+      <c r="E5" s="7" t="inlineStr">
+        <is>
+          <t>DURACIÓN</t>
+        </is>
+      </c>
+      <c r="F5" s="7" t="inlineStr">
+        <is>
+          <t>TIPO DE STORY</t>
+        </is>
+      </c>
+      <c r="G5" s="7" t="inlineStr">
+        <is>
+          <t>TIPO DE REEL</t>
+        </is>
+      </c>
+      <c r="H5" s="7" t="inlineStr">
+        <is>
+          <t>TIPO DE CARRUSEL</t>
+        </is>
+      </c>
+      <c r="I5" s="7" t="inlineStr">
+        <is>
+          <t>CANTIDAD DE SLIDES</t>
+        </is>
       </c>
       <c r="J5" s="7" t="inlineStr">
         <is>
-          <t>Cantidad de Slides</t>
+          <t>ANILLO</t>
         </is>
       </c>
       <c r="K5" s="7" t="inlineStr">
         <is>
-          <t>Tipo de Reel</t>
+          <t>PARA AD</t>
         </is>
       </c>
       <c r="L5" s="7" t="inlineStr">
         <is>
-          <t>Tipo de Carrusel</t>
+          <t>OBSERVACIONES ESTRATÉGICAS</t>
         </is>
       </c>
     </row>
@@ -4798,10 +4861,10 @@
     <row r="1000" ht="15.75" customHeight="1"/>
   </sheetData>
   <mergeCells count="4">
-    <mergeCell ref="A1:I1"/>
+    <mergeCell ref="A1:L1"/>
     <mergeCell ref="B2:D2"/>
-    <mergeCell ref="F2:I2"/>
-    <mergeCell ref="A3:I3"/>
+    <mergeCell ref="F2:L2"/>
+    <mergeCell ref="A3:L3"/>
   </mergeCells>
   <printOptions/>
   <dataValidations count="7">
@@ -4815,16 +4878,16 @@
       <formula1>"informativa,encuesta,caja_de_pregunta,micro_impacto"</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="G6:G105">
-      <formula1>"1,2,3,4,5"</formula1>
+      <formula1>"Talking head,UGC / testimonio,Tutorial / educativo,Trend / audio viral"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="H6:H105">
+      <formula1>"Educativo / tips,Storytelling,Antes / después,Listicle"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="I6:I105">
+      <formula1>"3,4,5,6,7,8,9,10"</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="J6:J105">
-      <formula1>"3,4,5,6,7,8,9,10"</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="K6:K105">
-      <formula1>"Talking head,UGC / testimonio,Tutorial / educativo,Trend / audio viral"</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="L6:L105">
-      <formula1>"Educativo / tips,Storytelling,Antes / después,Listicle"</formula1>
+      <formula1>"1,2,3,4,5"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins bottom="1.0" footer="0.0" header="0.0" left="0.75" right="0.75" top="1.0"/>
@@ -4846,10 +4909,13 @@
     <col customWidth="1" min="4" max="4" width="13.0"/>
     <col customWidth="1" min="5" max="5" width="11.0"/>
     <col customWidth="1" min="6" max="6" width="17.0"/>
-    <col customWidth="1" min="7" max="7" width="8.0"/>
-    <col customWidth="1" min="8" max="8" width="13.0"/>
-    <col customWidth="1" min="9" max="9" width="36.0"/>
-    <col customWidth="1" min="10" max="26" width="8.71"/>
+    <col customWidth="1" min="7" max="7" width="17.0"/>
+    <col customWidth="1" min="8" max="8" width="17.0"/>
+    <col customWidth="1" min="9" max="9" width="13.0"/>
+    <col customWidth="1" min="10" max="10" width="8.0"/>
+    <col customWidth="1" min="11" max="11" width="10.0"/>
+    <col customWidth="1" min="12" max="12" width="36.0"/>
+    <col min="13" max="26" width="9.0"/>
   </cols>
   <sheetData>
     <row r="1" ht="30.0" customHeight="1">
@@ -4891,46 +4957,64 @@
     </row>
     <row r="4" ht="6.0" customHeight="1"/>
     <row r="5" ht="27.75" customHeight="1">
-      <c r="A5" s="7" t="s">
-        <v>6</v>
-      </c>
-      <c r="B5" s="7" t="s">
-        <v>7</v>
-      </c>
-      <c r="C5" s="7" t="s">
-        <v>8</v>
-      </c>
-      <c r="D5" s="7" t="s">
-        <v>9</v>
-      </c>
-      <c r="E5" s="7" t="s">
-        <v>10</v>
-      </c>
-      <c r="F5" s="7" t="s">
-        <v>11</v>
-      </c>
-      <c r="G5" s="7" t="s">
-        <v>12</v>
-      </c>
-      <c r="H5" s="7" t="s">
-        <v>13</v>
-      </c>
-      <c r="I5" s="7" t="s">
-        <v>14</v>
+      <c r="A5" s="7" t="inlineStr">
+        <is>
+          <t>DÍA</t>
+        </is>
+      </c>
+      <c r="B5" s="7" t="inlineStr">
+        <is>
+          <t>FECHA DE PUBLICACIÓN</t>
+        </is>
+      </c>
+      <c r="C5" s="7" t="inlineStr">
+        <is>
+          <t>N°</t>
+        </is>
+      </c>
+      <c r="D5" s="7" t="inlineStr">
+        <is>
+          <t>TIPO DE PIEZA</t>
+        </is>
+      </c>
+      <c r="E5" s="7" t="inlineStr">
+        <is>
+          <t>DURACIÓN</t>
+        </is>
+      </c>
+      <c r="F5" s="7" t="inlineStr">
+        <is>
+          <t>TIPO DE STORY</t>
+        </is>
+      </c>
+      <c r="G5" s="7" t="inlineStr">
+        <is>
+          <t>TIPO DE REEL</t>
+        </is>
+      </c>
+      <c r="H5" s="7" t="inlineStr">
+        <is>
+          <t>TIPO DE CARRUSEL</t>
+        </is>
+      </c>
+      <c r="I5" s="7" t="inlineStr">
+        <is>
+          <t>CANTIDAD DE SLIDES</t>
+        </is>
       </c>
       <c r="J5" s="7" t="inlineStr">
         <is>
-          <t>Cantidad de Slides</t>
+          <t>ANILLO</t>
         </is>
       </c>
       <c r="K5" s="7" t="inlineStr">
         <is>
-          <t>Tipo de Reel</t>
+          <t>PARA AD</t>
         </is>
       </c>
       <c r="L5" s="7" t="inlineStr">
         <is>
-          <t>Tipo de Carrusel</t>
+          <t>OBSERVACIONES ESTRATÉGICAS</t>
         </is>
       </c>
     </row>
@@ -6211,10 +6295,10 @@
     <row r="1000" ht="15.75" customHeight="1"/>
   </sheetData>
   <mergeCells count="4">
-    <mergeCell ref="A1:I1"/>
+    <mergeCell ref="A1:L1"/>
     <mergeCell ref="B2:D2"/>
-    <mergeCell ref="F2:I2"/>
-    <mergeCell ref="A3:I3"/>
+    <mergeCell ref="F2:L2"/>
+    <mergeCell ref="A3:L3"/>
   </mergeCells>
   <printOptions/>
   <dataValidations count="7">
@@ -6228,16 +6312,16 @@
       <formula1>"informativa,encuesta,caja_de_pregunta,micro_impacto"</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="G6:G105">
-      <formula1>"1,2,3,4,5"</formula1>
+      <formula1>"Talking head,UGC / testimonio,Tutorial / educativo,Trend / audio viral"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="H6:H105">
+      <formula1>"Educativo / tips,Storytelling,Antes / después,Listicle"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="I6:I105">
+      <formula1>"3,4,5,6,7,8,9,10"</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="J6:J105">
-      <formula1>"3,4,5,6,7,8,9,10"</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="K6:K105">
-      <formula1>"Talking head,UGC / testimonio,Tutorial / educativo,Trend / audio viral"</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="L6:L105">
-      <formula1>"Educativo / tips,Storytelling,Antes / después,Listicle"</formula1>
+      <formula1>"1,2,3,4,5"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins bottom="1.0" footer="0.0" header="0.0" left="0.75" right="0.75" top="1.0"/>
@@ -6259,10 +6343,13 @@
     <col customWidth="1" min="4" max="4" width="13.0"/>
     <col customWidth="1" min="5" max="5" width="11.0"/>
     <col customWidth="1" min="6" max="6" width="17.0"/>
-    <col customWidth="1" min="7" max="7" width="8.0"/>
-    <col customWidth="1" min="8" max="8" width="13.0"/>
-    <col customWidth="1" min="9" max="9" width="36.0"/>
-    <col customWidth="1" min="10" max="26" width="8.71"/>
+    <col customWidth="1" min="7" max="7" width="17.0"/>
+    <col customWidth="1" min="8" max="8" width="17.0"/>
+    <col customWidth="1" min="9" max="9" width="13.0"/>
+    <col customWidth="1" min="10" max="10" width="8.0"/>
+    <col customWidth="1" min="11" max="11" width="10.0"/>
+    <col customWidth="1" min="12" max="12" width="36.0"/>
+    <col min="13" max="26" width="9.0"/>
   </cols>
   <sheetData>
     <row r="1" ht="30.0" customHeight="1">
@@ -6304,46 +6391,64 @@
     </row>
     <row r="4" ht="6.0" customHeight="1"/>
     <row r="5" ht="27.75" customHeight="1">
-      <c r="A5" s="7" t="s">
-        <v>6</v>
-      </c>
-      <c r="B5" s="7" t="s">
-        <v>7</v>
-      </c>
-      <c r="C5" s="7" t="s">
-        <v>8</v>
-      </c>
-      <c r="D5" s="7" t="s">
-        <v>9</v>
-      </c>
-      <c r="E5" s="7" t="s">
-        <v>10</v>
-      </c>
-      <c r="F5" s="7" t="s">
-        <v>11</v>
-      </c>
-      <c r="G5" s="7" t="s">
-        <v>12</v>
-      </c>
-      <c r="H5" s="7" t="s">
-        <v>13</v>
-      </c>
-      <c r="I5" s="7" t="s">
-        <v>14</v>
+      <c r="A5" s="7" t="inlineStr">
+        <is>
+          <t>DÍA</t>
+        </is>
+      </c>
+      <c r="B5" s="7" t="inlineStr">
+        <is>
+          <t>FECHA DE PUBLICACIÓN</t>
+        </is>
+      </c>
+      <c r="C5" s="7" t="inlineStr">
+        <is>
+          <t>N°</t>
+        </is>
+      </c>
+      <c r="D5" s="7" t="inlineStr">
+        <is>
+          <t>TIPO DE PIEZA</t>
+        </is>
+      </c>
+      <c r="E5" s="7" t="inlineStr">
+        <is>
+          <t>DURACIÓN</t>
+        </is>
+      </c>
+      <c r="F5" s="7" t="inlineStr">
+        <is>
+          <t>TIPO DE STORY</t>
+        </is>
+      </c>
+      <c r="G5" s="7" t="inlineStr">
+        <is>
+          <t>TIPO DE REEL</t>
+        </is>
+      </c>
+      <c r="H5" s="7" t="inlineStr">
+        <is>
+          <t>TIPO DE CARRUSEL</t>
+        </is>
+      </c>
+      <c r="I5" s="7" t="inlineStr">
+        <is>
+          <t>CANTIDAD DE SLIDES</t>
+        </is>
       </c>
       <c r="J5" s="7" t="inlineStr">
         <is>
-          <t>Cantidad de Slides</t>
+          <t>ANILLO</t>
         </is>
       </c>
       <c r="K5" s="7" t="inlineStr">
         <is>
-          <t>Tipo de Reel</t>
+          <t>PARA AD</t>
         </is>
       </c>
       <c r="L5" s="7" t="inlineStr">
         <is>
-          <t>Tipo de Carrusel</t>
+          <t>OBSERVACIONES ESTRATÉGICAS</t>
         </is>
       </c>
     </row>
@@ -7415,10 +7520,10 @@
     <row r="1000" ht="15.75" customHeight="1"/>
   </sheetData>
   <mergeCells count="4">
-    <mergeCell ref="A1:I1"/>
+    <mergeCell ref="A1:L1"/>
     <mergeCell ref="B2:D2"/>
-    <mergeCell ref="F2:I2"/>
-    <mergeCell ref="A3:I3"/>
+    <mergeCell ref="F2:L2"/>
+    <mergeCell ref="A3:L3"/>
   </mergeCells>
   <printOptions/>
   <dataValidations count="7">
@@ -7432,16 +7537,16 @@
       <formula1>"informativa,encuesta,caja_de_pregunta,micro_impacto"</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="G6:G105">
-      <formula1>"1,2,3,4,5"</formula1>
+      <formula1>"Talking head,UGC / testimonio,Tutorial / educativo,Trend / audio viral"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="H6:H105">
+      <formula1>"Educativo / tips,Storytelling,Antes / después,Listicle"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="I6:I105">
+      <formula1>"3,4,5,6,7,8,9,10"</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="J6:J105">
-      <formula1>"3,4,5,6,7,8,9,10"</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="K6:K105">
-      <formula1>"Talking head,UGC / testimonio,Tutorial / educativo,Trend / audio viral"</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="L6:L105">
-      <formula1>"Educativo / tips,Storytelling,Antes / después,Listicle"</formula1>
+      <formula1>"1,2,3,4,5"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins bottom="1.0" footer="0.0" header="0.0" left="0.75" right="0.75" top="1.0"/>

</xml_diff>